<commit_message>
Capture full workspace state
</commit_message>
<xml_diff>
--- a/4.Emails/07.24.26-Payment Plans CC Report 072426_FLYWIRE.xlsx
+++ b/4.Emails/07.24.26-Payment Plans CC Report 072426_FLYWIRE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\AP\Payment Plan Reports 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Renfrew\Workflow\4.Emails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BF1A5C8-C72E-4374-BAFC-054EFC24C880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322E196C-6566-4AE6-AE79-E422478BE071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3DE98709-DBE7-4539-AEBC-D09BE2D2BEC0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3DE98709-DBE7-4539-AEBC-D09BE2D2BEC0}"/>
   </bookViews>
   <sheets>
     <sheet name="PaymentsDetailedReport20260724_" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">PaymentsDetailedReport20260724_!$A$1:$K$4</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -95,10 +108,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,8 +247,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.14999847407452621"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -417,6 +438,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -557,7 +584,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -600,8 +627,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -624,8 +652,12 @@
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="33" borderId="0" xfId="42" applyFont="1" applyFill="1"/>
+    <xf numFmtId="40" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -653,6 +685,7 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="42" builtinId="3"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -999,23 +1032,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB26CC7F-1DED-4E74-82B7-3FD91E9D1929}">
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="22.85546875" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" customWidth="1"/>
-    <col min="11" max="11" width="25.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.88671875" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.88671875" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="7" max="7" width="20.44140625" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="22.88671875" customWidth="1"/>
+    <col min="10" max="10" width="18.33203125" customWidth="1"/>
+    <col min="11" max="11" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +1083,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1084,8 +1117,36 @@
       <c r="K2" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="M2" s="8">
+        <f>F2</f>
+        <v>303.13</v>
+      </c>
+      <c r="N2" s="9" t="str">
+        <f>H2&amp;": "&amp;I2&amp;"- "&amp;J2</f>
+        <v>135922: Alexis Young- David Young</v>
+      </c>
+      <c r="O2" s="10" t="str">
+        <f>Q2&amp;R2</f>
+        <v>VS-6877</v>
+      </c>
+      <c r="P2" s="11" t="str">
+        <f>LEFT(S2,4)</f>
+        <v>Visa</v>
+      </c>
+      <c r="Q2" s="11" t="str">
+        <f>IF(P2="Visa","VS-",IF(P2="Mast","MC-",IF(P2="Disc","DIS-",IF(P2="amer","AMEX-"))))</f>
+        <v>VS-</v>
+      </c>
+      <c r="R2" s="11" t="str">
+        <f>RIGHT(S2,4)</f>
+        <v>6877</v>
+      </c>
+      <c r="S2" s="11" t="str">
+        <f>MID(C2,8,(LEN(C2)-5))</f>
+        <v>Visa - 6877</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1098,7 +1159,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>21</v>
       </c>
@@ -1118,7 +1179,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1131,7 +1192,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1144,7 +1205,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1157,7 +1218,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1170,7 +1231,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1183,7 +1244,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1196,7 +1257,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1209,7 +1270,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1222,7 +1283,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>

</xml_diff>